<commit_message>
E4-E6 od nowa: poprawne scenariusze, wyniki formuł i tabele danych
</commit_message>
<xml_diff>
--- a/E4-E6/TI.1_Excel.E4+E5+E6_PlikRoboczy.xlsx
+++ b/E4-E6/TI.1_Excel.E4+E5+E6_PlikRoboczy.xlsx
@@ -1467,6 +1467,12 @@
 Dlatego użyto INDEKS + PODAJ.POZYCJĘ.</t>
       </text>
     </comment>
+    <comment ref="I57" authorId="0" shapeId="0">
+      <text>
+        <t>Przy wadze 100 g (stan po E4) ZYSK = -2 019 €.
+Po Szukaj wyniku (90,386 g) ZYSK = 10 000 €.</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -1880,7 +1886,7 @@
       </c>
       <c r="C7" s="102">
         <f>IF(C31&lt;&gt;0,I48/C31,"Nie można dzielić przez 0")</f>
-        <v/>
+        <v>1.94827586206897</v>
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
@@ -2011,7 +2017,7 @@
       </c>
       <c r="H13" s="8">
         <f>1-SUM(D13:G13)</f>
-        <v/>
+        <v>0.3</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -2104,25 +2110,25 @@
           <t>Liczba parówek</t>
         </is>
       </c>
-      <c r="D18" s="6">
+      <c r="D18" s="6" t="str">
         <f>D12</f>
-        <v/>
-      </c>
-      <c r="E18" s="6">
+        <v>Smocze sadło</v>
+      </c>
+      <c r="E18" s="6" t="str">
         <f>E12</f>
-        <v/>
-      </c>
-      <c r="F18" s="6">
+        <v>Mrówcze mięso</v>
+      </c>
+      <c r="F18" s="6" t="str">
         <f>F12</f>
-        <v/>
-      </c>
-      <c r="G18" s="6">
+        <v>Makula-tura</v>
+      </c>
+      <c r="G18" s="6" t="str">
         <f>G12</f>
-        <v/>
-      </c>
-      <c r="H18" s="7">
+        <v>Magic Stufff</v>
+      </c>
+      <c r="H18" s="7" t="str">
         <f>H12</f>
-        <v/>
+        <v>Woda</v>
       </c>
       <c r="I18" s="86" t="n"/>
       <c r="J18" s="86" t="n"/>
@@ -2149,23 +2155,23 @@
       </c>
       <c r="D19" s="107">
         <f>$C19*$C$9/1000*D$13</f>
-        <v/>
+        <v>108.463513545941</v>
       </c>
       <c r="E19" s="108">
         <f>$C19*$C$9/1000*E$13</f>
-        <v/>
+        <v>72.3090090306273</v>
       </c>
       <c r="F19" s="108">
         <f>$C19*$C$9/1000*F$13</f>
-        <v/>
+        <v>54.2317567729705</v>
       </c>
       <c r="G19" s="108">
         <f>$C19*$C$9/1000*G$13</f>
-        <v/>
+        <v>18.0772522576568</v>
       </c>
       <c r="H19" s="108">
         <f>$C19*$C$9/1000*H$13</f>
-        <v/>
+        <v>108.463513545941</v>
       </c>
       <c r="I19" s="109" t="n"/>
       <c r="J19" s="86" t="n"/>
@@ -2192,23 +2198,23 @@
       </c>
       <c r="D20" s="108">
         <f>$C20*$C$9/1000*D$13</f>
-        <v/>
+        <v>130.156216255129</v>
       </c>
       <c r="E20" s="108">
         <f>$C20*$C$9/1000*E$13</f>
-        <v/>
+        <v>86.7708108367528</v>
       </c>
       <c r="F20" s="108">
         <f>$C20*$C$9/1000*F$13</f>
-        <v/>
+        <v>65.0781081275646</v>
       </c>
       <c r="G20" s="108">
         <f>$C20*$C$9/1000*G$13</f>
-        <v/>
+        <v>21.6927027091882</v>
       </c>
       <c r="H20" s="108">
         <f>$C20*$C$9/1000*H$13</f>
-        <v/>
+        <v>130.156216255129</v>
       </c>
       <c r="I20" s="109" t="n"/>
       <c r="J20" s="86" t="n"/>
@@ -2235,23 +2241,23 @@
       </c>
       <c r="D21" s="108">
         <f>$C21*$C$9/1000*D$13</f>
-        <v/>
+        <v>151.848918964317</v>
       </c>
       <c r="E21" s="108">
         <f>$C21*$C$9/1000*E$13</f>
-        <v/>
+        <v>101.232612642878</v>
       </c>
       <c r="F21" s="108">
         <f>$C21*$C$9/1000*F$13</f>
-        <v/>
+        <v>75.9244594821587</v>
       </c>
       <c r="G21" s="108">
         <f>$C21*$C$9/1000*G$13</f>
-        <v/>
+        <v>25.3081531607196</v>
       </c>
       <c r="H21" s="108">
         <f>$C21*$C$9/1000*H$13</f>
-        <v/>
+        <v>151.848918964317</v>
       </c>
       <c r="I21" s="109" t="n"/>
       <c r="J21" s="86" t="n"/>
@@ -2278,23 +2284,23 @@
       </c>
       <c r="D22" s="108">
         <f>$C22*$C$9/1000*D$13</f>
-        <v/>
+        <v>173.541621673506</v>
       </c>
       <c r="E22" s="108">
         <f>$C22*$C$9/1000*E$13</f>
-        <v/>
+        <v>115.694414449004</v>
       </c>
       <c r="F22" s="108">
         <f>$C22*$C$9/1000*F$13</f>
-        <v/>
+        <v>86.7708108367528</v>
       </c>
       <c r="G22" s="108">
         <f>$C22*$C$9/1000*G$13</f>
-        <v/>
+        <v>28.9236036122509</v>
       </c>
       <c r="H22" s="108">
         <f>$C22*$C$9/1000*H$13</f>
-        <v/>
+        <v>173.541621673506</v>
       </c>
       <c r="I22" s="109" t="n"/>
       <c r="J22" s="86" t="n"/>
@@ -2321,23 +2327,23 @@
       </c>
       <c r="D23" s="108">
         <f>$C23*$C$9/1000*D$13</f>
-        <v/>
+        <v>195.234324382694</v>
       </c>
       <c r="E23" s="108">
         <f>$C23*$C$9/1000*E$13</f>
-        <v/>
+        <v>130.156216255129</v>
       </c>
       <c r="F23" s="108">
         <f>$C23*$C$9/1000*F$13</f>
-        <v/>
+        <v>97.6171621913469</v>
       </c>
       <c r="G23" s="108">
         <f>$C23*$C$9/1000*G$13</f>
-        <v/>
+        <v>32.5390540637823</v>
       </c>
       <c r="H23" s="108">
         <f>$C23*$C$9/1000*H$13</f>
-        <v/>
+        <v>195.234324382694</v>
       </c>
       <c r="I23" s="109" t="n"/>
       <c r="J23" s="86" t="n"/>
@@ -2364,23 +2370,23 @@
       </c>
       <c r="D24" s="108">
         <f>$C24*$C$9/1000*D$13</f>
-        <v/>
+        <v>216.927027091882</v>
       </c>
       <c r="E24" s="108">
         <f>$C24*$C$9/1000*E$13</f>
-        <v/>
+        <v>144.618018061255</v>
       </c>
       <c r="F24" s="108">
         <f>$C24*$C$9/1000*F$13</f>
-        <v/>
+        <v>108.463513545941</v>
       </c>
       <c r="G24" s="108">
         <f>$C24*$C$9/1000*G$13</f>
-        <v/>
+        <v>36.1545045153137</v>
       </c>
       <c r="H24" s="108">
         <f>$C24*$C$9/1000*H$13</f>
-        <v/>
+        <v>216.927027091882</v>
       </c>
       <c r="I24" s="109" t="n"/>
       <c r="J24" s="86" t="n"/>
@@ -2407,23 +2413,23 @@
       </c>
       <c r="D25" s="108">
         <f>$C25*$C$9/1000*D$13</f>
-        <v/>
+        <v>43.3854054183764</v>
       </c>
       <c r="E25" s="108">
         <f>$C25*$C$9/1000*E$13</f>
-        <v/>
+        <v>28.9236036122509</v>
       </c>
       <c r="F25" s="108">
         <f>$C25*$C$9/1000*F$13</f>
-        <v/>
+        <v>21.6927027091882</v>
       </c>
       <c r="G25" s="108">
         <f>$C25*$C$9/1000*G$13</f>
-        <v/>
+        <v>7.23090090306273</v>
       </c>
       <c r="H25" s="108">
         <f>$C25*$C$9/1000*H$13</f>
-        <v/>
+        <v>43.3854054183764</v>
       </c>
       <c r="I25" s="109" t="n"/>
       <c r="J25" s="86" t="n"/>
@@ -2450,23 +2456,23 @@
       </c>
       <c r="D26" s="108">
         <f>$C26*$C$9/1000*D$13</f>
-        <v/>
+        <v>21.6927027091882</v>
       </c>
       <c r="E26" s="108">
         <f>$C26*$C$9/1000*E$13</f>
-        <v/>
+        <v>14.4618018061255</v>
       </c>
       <c r="F26" s="108">
         <f>$C26*$C$9/1000*F$13</f>
-        <v/>
+        <v>10.8463513545941</v>
       </c>
       <c r="G26" s="108">
         <f>$C26*$C$9/1000*G$13</f>
-        <v/>
+        <v>3.61545045153137</v>
       </c>
       <c r="H26" s="108">
         <f>$C26*$C$9/1000*H$13</f>
-        <v/>
+        <v>21.6927027091882</v>
       </c>
       <c r="I26" s="109" t="n"/>
       <c r="J26" s="86" t="n"/>
@@ -2493,23 +2499,23 @@
       </c>
       <c r="D27" s="108">
         <f>$C27*$C$9/1000*D$13</f>
-        <v/>
+        <v>108.463513545941</v>
       </c>
       <c r="E27" s="108">
         <f>$C27*$C$9/1000*E$13</f>
-        <v/>
+        <v>72.3090090306273</v>
       </c>
       <c r="F27" s="108">
         <f>$C27*$C$9/1000*F$13</f>
-        <v/>
+        <v>54.2317567729705</v>
       </c>
       <c r="G27" s="108">
         <f>$C27*$C$9/1000*G$13</f>
-        <v/>
+        <v>18.0772522576568</v>
       </c>
       <c r="H27" s="108">
         <f>$C27*$C$9/1000*H$13</f>
-        <v/>
+        <v>108.463513545941</v>
       </c>
       <c r="I27" s="109" t="n"/>
       <c r="J27" s="86" t="n"/>
@@ -2536,23 +2542,23 @@
       </c>
       <c r="D28" s="108">
         <f>$C28*$C$9/1000*D$13</f>
-        <v/>
+        <v>130.156216255129</v>
       </c>
       <c r="E28" s="108">
         <f>$C28*$C$9/1000*E$13</f>
-        <v/>
+        <v>86.7708108367528</v>
       </c>
       <c r="F28" s="108">
         <f>$C28*$C$9/1000*F$13</f>
-        <v/>
+        <v>65.0781081275646</v>
       </c>
       <c r="G28" s="108">
         <f>$C28*$C$9/1000*G$13</f>
-        <v/>
+        <v>21.6927027091882</v>
       </c>
       <c r="H28" s="108">
         <f>$C28*$C$9/1000*H$13</f>
-        <v/>
+        <v>130.156216255129</v>
       </c>
       <c r="I28" s="109" t="n"/>
       <c r="J28" s="86" t="n"/>
@@ -2579,23 +2585,23 @@
       </c>
       <c r="D29" s="108">
         <f>$C29*$C$9/1000*D$13</f>
-        <v/>
+        <v>151.848918964317</v>
       </c>
       <c r="E29" s="108">
         <f>$C29*$C$9/1000*E$13</f>
-        <v/>
+        <v>101.232612642878</v>
       </c>
       <c r="F29" s="108">
         <f>$C29*$C$9/1000*F$13</f>
-        <v/>
+        <v>75.9244594821587</v>
       </c>
       <c r="G29" s="108">
         <f>$C29*$C$9/1000*G$13</f>
-        <v/>
+        <v>25.3081531607196</v>
       </c>
       <c r="H29" s="108">
         <f>$C29*$C$9/1000*H$13</f>
-        <v/>
+        <v>151.848918964317</v>
       </c>
       <c r="I29" s="109" t="n"/>
       <c r="J29" s="86" t="n"/>
@@ -2622,23 +2628,23 @@
       </c>
       <c r="D30" s="108">
         <f>$C30*$C$9/1000*D$13</f>
-        <v/>
+        <v>141.002567609723</v>
       </c>
       <c r="E30" s="108">
         <f>$C30*$C$9/1000*E$13</f>
-        <v/>
+        <v>94.0017117398156</v>
       </c>
       <c r="F30" s="108">
         <f>$C30*$C$9/1000*F$13</f>
-        <v/>
+        <v>70.5012838048617</v>
       </c>
       <c r="G30" s="108">
         <f>$C30*$C$9/1000*G$13</f>
-        <v/>
+        <v>23.5004279349539</v>
       </c>
       <c r="H30" s="108">
         <f>$C30*$C$9/1000*H$13</f>
-        <v/>
+        <v>141.002567609723</v>
       </c>
       <c r="I30" s="109" t="n"/>
       <c r="J30" s="86" t="n"/>
@@ -2662,27 +2668,27 @@
       </c>
       <c r="C31" s="44">
         <f>SUM(C19:C30)</f>
-        <v/>
+        <v>58000</v>
       </c>
       <c r="D31" s="45">
         <f>SUM(D19:D30)</f>
-        <v/>
+        <v>1572.72094641614</v>
       </c>
       <c r="E31" s="45">
         <f>SUM(E19:E30)</f>
-        <v/>
+        <v>1048.4806309441</v>
       </c>
       <c r="F31" s="45">
         <f>SUM(F19:F30)</f>
-        <v/>
+        <v>786.360473208072</v>
       </c>
       <c r="G31" s="45">
         <f>SUM(G19:G30)</f>
-        <v/>
+        <v>262.120157736024</v>
       </c>
       <c r="H31" s="45">
         <f>SUM(H19:H30)</f>
-        <v/>
+        <v>1572.72094641614</v>
       </c>
       <c r="I31" s="86" t="n"/>
       <c r="J31" s="86" t="n"/>
@@ -2744,30 +2750,30 @@
       <c r="H34" s="16" t="n"/>
     </row>
     <row r="35" ht="30" customHeight="1">
-      <c r="B35" s="88">
+      <c r="B35" s="88" t="str">
         <f>B18</f>
-        <v/>
+        <v>Miesiąc</v>
       </c>
       <c r="C35" s="16" t="n"/>
-      <c r="D35" s="6">
+      <c r="D35" s="6" t="str">
         <f>D18</f>
-        <v/>
-      </c>
-      <c r="E35" s="6">
+        <v>Smocze sadło</v>
+      </c>
+      <c r="E35" s="6" t="str">
         <f>E18</f>
-        <v/>
-      </c>
-      <c r="F35" s="6">
+        <v>Mrówcze mięso</v>
+      </c>
+      <c r="F35" s="6" t="str">
         <f>F18</f>
-        <v/>
-      </c>
-      <c r="G35" s="6">
+        <v>Makula-tura</v>
+      </c>
+      <c r="G35" s="6" t="str">
         <f>G18</f>
-        <v/>
-      </c>
-      <c r="H35" s="53">
+        <v>Magic Stufff</v>
+      </c>
+      <c r="H35" s="53" t="str">
         <f>H18</f>
-        <v/>
+        <v>Woda</v>
       </c>
       <c r="I35" s="54" t="inlineStr">
         <is>
@@ -2776,375 +2782,375 @@
       </c>
     </row>
     <row r="36">
-      <c r="B36" s="41">
+      <c r="B36" s="41" t="str">
         <f>B19</f>
-        <v/>
+        <v>Sty</v>
       </c>
       <c r="C36" s="46" t="n"/>
       <c r="D36" s="61">
         <f>D19*D$14</f>
-        <v/>
+        <v>1626.95270318912</v>
       </c>
       <c r="E36" s="57">
         <f>E19*E$14</f>
-        <v/>
+        <v>5784.72072245019</v>
       </c>
       <c r="F36" s="57">
         <f>F19*F$14</f>
-        <v/>
+        <v>325.390540637823</v>
       </c>
       <c r="G36" s="57">
         <f>G19*G$14</f>
-        <v/>
+        <v>45.1931306441421</v>
       </c>
       <c r="H36" s="58">
         <f>H19*H$14</f>
-        <v/>
+        <v>10.8463513545941</v>
       </c>
       <c r="I36" s="47">
         <f>SUM(D36:H36)</f>
-        <v/>
+        <v>7793.10344827586</v>
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="41">
+      <c r="B37" s="41" t="str">
         <f>B20</f>
-        <v/>
+        <v>Lut</v>
       </c>
       <c r="C37" s="17" t="n"/>
       <c r="D37" s="59">
         <f>D20*D$14</f>
-        <v/>
+        <v>1952.34324382694</v>
       </c>
       <c r="E37" s="59">
         <f>E20*E$14</f>
-        <v/>
+        <v>6941.66486694023</v>
       </c>
       <c r="F37" s="59">
         <f>F20*F$14</f>
-        <v/>
+        <v>390.468648765388</v>
       </c>
       <c r="G37" s="59">
         <f>G20*G$14</f>
-        <v/>
+        <v>54.2317567729705</v>
       </c>
       <c r="H37" s="60">
         <f>H20*H$14</f>
-        <v/>
+        <v>13.0156216255129</v>
       </c>
       <c r="I37" s="19">
         <f>SUM(D37:H37)</f>
-        <v/>
+        <v>9351.72413793103</v>
       </c>
     </row>
     <row r="38">
-      <c r="B38" s="41">
+      <c r="B38" s="41" t="str">
         <f>B21</f>
-        <v/>
+        <v>Mar</v>
       </c>
       <c r="C38" s="17" t="n"/>
       <c r="D38" s="59">
         <f>D21*D$14</f>
-        <v/>
+        <v>2277.73378446476</v>
       </c>
       <c r="E38" s="59">
         <f>E21*E$14</f>
-        <v/>
+        <v>8098.60901143026</v>
       </c>
       <c r="F38" s="59">
         <f>F21*F$14</f>
-        <v/>
+        <v>455.546756892952</v>
       </c>
       <c r="G38" s="59">
         <f>G21*G$14</f>
-        <v/>
+        <v>63.2703829017989</v>
       </c>
       <c r="H38" s="60">
         <f>H21*H$14</f>
-        <v/>
+        <v>15.1848918964317</v>
       </c>
       <c r="I38" s="19">
         <f>SUM(D38:H38)</f>
-        <v/>
+        <v>10910.3448275862</v>
       </c>
     </row>
     <row r="39">
-      <c r="B39" s="41">
+      <c r="B39" s="41" t="str">
         <f>B22</f>
-        <v/>
+        <v>Kwi</v>
       </c>
       <c r="C39" s="17" t="n"/>
       <c r="D39" s="59">
         <f>D22*D$14</f>
-        <v/>
+        <v>2603.12432510258</v>
       </c>
       <c r="E39" s="59">
         <f>E22*E$14</f>
-        <v/>
+        <v>9255.5531559203</v>
       </c>
       <c r="F39" s="59">
         <f>F22*F$14</f>
-        <v/>
+        <v>520.624865020517</v>
       </c>
       <c r="G39" s="59">
         <f>G22*G$14</f>
-        <v/>
+        <v>72.3090090306273</v>
       </c>
       <c r="H39" s="60">
         <f>H22*H$14</f>
-        <v/>
+        <v>17.3541621673506</v>
       </c>
       <c r="I39" s="19">
         <f>SUM(D39:H39)</f>
-        <v/>
+        <v>12468.9655172414</v>
       </c>
     </row>
     <row r="40">
-      <c r="B40" s="41">
+      <c r="B40" s="41" t="str">
         <f>B23</f>
-        <v/>
+        <v>Maj</v>
       </c>
       <c r="C40" s="17" t="n"/>
       <c r="D40" s="59">
         <f>D23*D$14</f>
-        <v/>
+        <v>2928.51486574041</v>
       </c>
       <c r="E40" s="59">
         <f>E23*E$14</f>
-        <v/>
+        <v>10412.4973004103</v>
       </c>
       <c r="F40" s="59">
         <f>F23*F$14</f>
-        <v/>
+        <v>585.702973148082</v>
       </c>
       <c r="G40" s="59">
         <f>G23*G$14</f>
-        <v/>
+        <v>81.3476351594558</v>
       </c>
       <c r="H40" s="60">
         <f>H23*H$14</f>
-        <v/>
+        <v>19.5234324382694</v>
       </c>
       <c r="I40" s="19">
         <f>SUM(D40:H40)</f>
-        <v/>
+        <v>14027.5862068966</v>
       </c>
     </row>
     <row r="41">
-      <c r="B41" s="41">
+      <c r="B41" s="41" t="str">
         <f>B24</f>
-        <v/>
+        <v>Cze</v>
       </c>
       <c r="C41" s="17" t="n"/>
       <c r="D41" s="59">
         <f>D24*D$14</f>
-        <v/>
+        <v>3253.90540637823</v>
       </c>
       <c r="E41" s="59">
         <f>E24*E$14</f>
-        <v/>
+        <v>11569.4414449004</v>
       </c>
       <c r="F41" s="59">
         <f>F24*F$14</f>
-        <v/>
+        <v>650.781081275646</v>
       </c>
       <c r="G41" s="59">
         <f>G24*G$14</f>
-        <v/>
+        <v>90.3862612882842</v>
       </c>
       <c r="H41" s="60">
         <f>H24*H$14</f>
-        <v/>
+        <v>21.6927027091882</v>
       </c>
       <c r="I41" s="19">
         <f>SUM(D41:H41)</f>
-        <v/>
+        <v>15586.2068965517</v>
       </c>
     </row>
     <row r="42">
-      <c r="B42" s="41">
+      <c r="B42" s="41" t="str">
         <f>B25</f>
-        <v/>
+        <v>Lip</v>
       </c>
       <c r="C42" s="17" t="n"/>
       <c r="D42" s="59">
         <f>D25*D$14</f>
-        <v/>
+        <v>650.781081275646</v>
       </c>
       <c r="E42" s="59">
         <f>E25*E$14</f>
-        <v/>
+        <v>2313.88828898008</v>
       </c>
       <c r="F42" s="59">
         <f>F25*F$14</f>
-        <v/>
+        <v>130.156216255129</v>
       </c>
       <c r="G42" s="59">
         <f>G25*G$14</f>
-        <v/>
+        <v>18.0772522576568</v>
       </c>
       <c r="H42" s="60">
         <f>H25*H$14</f>
-        <v/>
+        <v>4.33854054183764</v>
       </c>
       <c r="I42" s="19">
         <f>SUM(D42:H42)</f>
-        <v/>
+        <v>3117.24137931034</v>
       </c>
     </row>
     <row r="43">
-      <c r="B43" s="41">
+      <c r="B43" s="41" t="str">
         <f>B26</f>
-        <v/>
+        <v>Sie</v>
       </c>
       <c r="C43" s="17" t="n"/>
       <c r="D43" s="59">
         <f>D26*D$14</f>
-        <v/>
+        <v>325.390540637823</v>
       </c>
       <c r="E43" s="59">
         <f>E26*E$14</f>
-        <v/>
+        <v>1156.94414449004</v>
       </c>
       <c r="F43" s="59">
         <f>F26*F$14</f>
-        <v/>
+        <v>65.0781081275646</v>
       </c>
       <c r="G43" s="59">
         <f>G26*G$14</f>
-        <v/>
+        <v>9.03862612882842</v>
       </c>
       <c r="H43" s="60">
         <f>H26*H$14</f>
-        <v/>
+        <v>2.16927027091882</v>
       </c>
       <c r="I43" s="19">
         <f>SUM(D43:H43)</f>
-        <v/>
+        <v>1558.62068965517</v>
       </c>
     </row>
     <row r="44">
-      <c r="B44" s="41">
+      <c r="B44" s="41" t="str">
         <f>B27</f>
-        <v/>
+        <v>Wrz</v>
       </c>
       <c r="C44" s="17" t="n"/>
       <c r="D44" s="59">
         <f>D27*D$14</f>
-        <v/>
+        <v>1626.95270318912</v>
       </c>
       <c r="E44" s="59">
         <f>E27*E$14</f>
-        <v/>
+        <v>5784.72072245019</v>
       </c>
       <c r="F44" s="59">
         <f>F27*F$14</f>
-        <v/>
+        <v>325.390540637823</v>
       </c>
       <c r="G44" s="59">
         <f>G27*G$14</f>
-        <v/>
+        <v>45.1931306441421</v>
       </c>
       <c r="H44" s="60">
         <f>H27*H$14</f>
-        <v/>
+        <v>10.8463513545941</v>
       </c>
       <c r="I44" s="19">
         <f>SUM(D44:H44)</f>
-        <v/>
+        <v>7793.10344827586</v>
       </c>
     </row>
     <row r="45">
-      <c r="B45" s="41">
+      <c r="B45" s="41" t="str">
         <f>B28</f>
-        <v/>
+        <v>Paź</v>
       </c>
       <c r="C45" s="17" t="n"/>
       <c r="D45" s="59">
         <f>D28*D$14</f>
-        <v/>
+        <v>1952.34324382694</v>
       </c>
       <c r="E45" s="59">
         <f>E28*E$14</f>
-        <v/>
+        <v>6941.66486694023</v>
       </c>
       <c r="F45" s="59">
         <f>F28*F$14</f>
-        <v/>
+        <v>390.468648765388</v>
       </c>
       <c r="G45" s="59">
         <f>G28*G$14</f>
-        <v/>
+        <v>54.2317567729705</v>
       </c>
       <c r="H45" s="60">
         <f>H28*H$14</f>
-        <v/>
+        <v>13.0156216255129</v>
       </c>
       <c r="I45" s="19">
         <f>SUM(D45:H45)</f>
-        <v/>
+        <v>9351.72413793103</v>
       </c>
     </row>
     <row r="46">
-      <c r="B46" s="41">
+      <c r="B46" s="41" t="str">
         <f>B29</f>
-        <v/>
+        <v>Lis</v>
       </c>
       <c r="C46" s="17" t="n"/>
       <c r="D46" s="59">
         <f>D29*D$14</f>
-        <v/>
+        <v>2277.73378446476</v>
       </c>
       <c r="E46" s="59">
         <f>E29*E$14</f>
-        <v/>
+        <v>8098.60901143026</v>
       </c>
       <c r="F46" s="59">
         <f>F29*F$14</f>
-        <v/>
+        <v>455.546756892952</v>
       </c>
       <c r="G46" s="59">
         <f>G29*G$14</f>
-        <v/>
+        <v>63.2703829017989</v>
       </c>
       <c r="H46" s="60">
         <f>H29*H$14</f>
-        <v/>
+        <v>15.1848918964317</v>
       </c>
       <c r="I46" s="19">
         <f>SUM(D46:H46)</f>
-        <v/>
+        <v>10910.3448275862</v>
       </c>
     </row>
     <row r="47">
-      <c r="B47" s="41">
+      <c r="B47" s="41" t="str">
         <f>B30</f>
-        <v/>
+        <v>Gru</v>
       </c>
       <c r="C47" s="17" t="n"/>
       <c r="D47" s="59">
         <f>D30*D$14</f>
-        <v/>
+        <v>2115.03851414585</v>
       </c>
       <c r="E47" s="59">
         <f>E30*E$14</f>
-        <v/>
+        <v>7520.13693918524</v>
       </c>
       <c r="F47" s="59">
         <f>F30*F$14</f>
-        <v/>
+        <v>423.00770282917</v>
       </c>
       <c r="G47" s="59">
         <f>G30*G$14</f>
-        <v/>
+        <v>58.7510698373847</v>
       </c>
       <c r="H47" s="60">
         <f>H30*H$14</f>
-        <v/>
+        <v>14.1002567609723</v>
       </c>
       <c r="I47" s="19">
         <f>SUM(D47:H47)</f>
-        <v/>
+        <v>10131.0344827586</v>
       </c>
     </row>
     <row r="48" ht="15.75" customHeight="1" thickBot="1">
@@ -3156,27 +3162,27 @@
       <c r="C48" s="49" t="n"/>
       <c r="D48" s="50">
         <f>SUM(D36:D47)</f>
-        <v/>
+        <v>23590.8141962422</v>
       </c>
       <c r="E48" s="50">
         <f>SUM(E36:E47)</f>
-        <v/>
+        <v>83878.4504755277</v>
       </c>
       <c r="F48" s="50">
         <f>SUM(F36:F47)</f>
-        <v/>
+        <v>4718.16283924843</v>
       </c>
       <c r="G48" s="51">
         <f>SUM(G36:G47)</f>
-        <v/>
+        <v>655.30039434006</v>
       </c>
       <c r="H48" s="51">
         <f>SUM(H36:H47)</f>
-        <v/>
+        <v>157.272094641614</v>
       </c>
       <c r="I48" s="52">
         <f>SUM(I36:I47)</f>
-        <v/>
+        <v>113000</v>
       </c>
       <c r="J48" s="18" t="inlineStr">
         <is>
@@ -3220,7 +3226,7 @@
       <c r="C51" s="12" t="n"/>
       <c r="D51" s="62">
         <f>MAX(I36:I47)</f>
-        <v/>
+        <v>15586.2068965517</v>
       </c>
       <c r="F51" s="78" t="n"/>
       <c r="G51" s="79" t="n"/>
@@ -3231,7 +3237,7 @@
       </c>
       <c r="I51" s="81">
         <f>C31*C6</f>
-        <v/>
+        <v>174000</v>
       </c>
       <c r="J51" t="inlineStr">
         <is>
@@ -3251,9 +3257,9 @@
         </is>
       </c>
       <c r="C52" s="12" t="n"/>
-      <c r="D52" s="63">
+      <c r="D52" s="63" t="str">
         <f>INDEX(B36:B47,MATCH(D51,I36:I47,0))</f>
-        <v/>
+        <v>Cze</v>
       </c>
       <c r="F52" s="69" t="n"/>
       <c r="G52" s="70" t="n"/>
@@ -3264,7 +3270,7 @@
       </c>
       <c r="I52" s="72">
         <f>I48</f>
-        <v/>
+        <v>113000</v>
       </c>
       <c r="J52" t="inlineStr">
         <is>
@@ -3286,7 +3292,7 @@
       <c r="C53" s="12" t="n"/>
       <c r="D53" s="63">
         <f>VLOOKUP(D52,B19:C30,2,0)</f>
-        <v/>
+        <v>8000</v>
       </c>
       <c r="F53" s="73" t="n"/>
       <c r="G53" s="65" t="n"/>
@@ -3297,7 +3303,7 @@
       </c>
       <c r="I53" s="74">
         <f>12*C8</f>
-        <v/>
+        <v>36000</v>
       </c>
       <c r="J53" t="inlineStr">
         <is>
@@ -3315,7 +3321,7 @@
       </c>
       <c r="I54" s="77">
         <f>I48+I53</f>
-        <v/>
+        <v>149000</v>
       </c>
       <c r="J54" t="inlineStr">
         <is>
@@ -3333,7 +3339,7 @@
       </c>
       <c r="I55" s="67">
         <f>I51-I54</f>
-        <v/>
+        <v>25000</v>
       </c>
       <c r="J55" t="inlineStr">
         <is>
@@ -3368,7 +3374,7 @@
       </c>
       <c r="I57" s="35">
         <f>I55-I56</f>
-        <v/>
+        <v>10000</v>
       </c>
       <c r="J57" t="inlineStr">
         <is>
@@ -3414,46 +3420,46 @@
       </c>
       <c r="C61" s="90">
         <f>I57</f>
-        <v/>
+        <v>10000</v>
       </c>
       <c r="E61" s="22">
         <f>I57</f>
-        <v/>
+        <v>10000</v>
       </c>
       <c r="F61" s="23" t="n">
         <v>70</v>
       </c>
       <c r="G61" s="23">
         <f>F61+5</f>
-        <v/>
+        <v>75</v>
       </c>
       <c r="H61" s="24">
         <f>G61+5</f>
-        <v/>
+        <v>80</v>
       </c>
       <c r="I61" s="23">
         <f>H61+5</f>
-        <v/>
+        <v>85</v>
       </c>
       <c r="J61" s="23">
         <f>I61+5</f>
-        <v/>
+        <v>90</v>
       </c>
       <c r="K61" s="23">
         <f>J61+5</f>
-        <v/>
+        <v>95</v>
       </c>
       <c r="L61" s="23">
         <f>K61+5</f>
-        <v/>
+        <v>100</v>
       </c>
       <c r="M61" s="23">
         <f>L61+5</f>
-        <v/>
+        <v>105</v>
       </c>
       <c r="N61" s="25">
         <f>M61+5</f>
-        <v/>
+        <v>110</v>
       </c>
     </row>
     <row r="62">
@@ -3461,7 +3467,7 @@
         <v>85</v>
       </c>
       <c r="C62" s="92">
-        <f t="dataTable" ref="C62:C82" dt2D="0" dtr="0" r1="$C$9"/>
+        <f t="dataTable" ref="C62:C82" dt2D="0" dtr="0" r1="$C$9" ca="1"/>
         <v>16733.85</v>
       </c>
       <c r="E62" s="26" t="n">
@@ -3469,7 +3475,7 @@
       </c>
       <c r="F62" s="27">
         <f t="dataTable" ref="F62:N72" dt2D="1" dtr="1" r1="$E$14" r2="$C$6" ca="1"/>
-        <v>-8515.19</v>
+        <v>-8515.19369055904</v>
       </c>
       <c r="G62" s="27" t="n">
         <v>-13757.59684528</v>
@@ -3499,14 +3505,14 @@
     <row r="63">
       <c r="B63" s="91">
         <f>B62+1</f>
-        <v/>
+        <v>86</v>
       </c>
       <c r="C63" s="92" t="n">
         <v>15483.66</v>
       </c>
       <c r="E63" s="26">
         <f>E62+0.1</f>
-        <v/>
+        <v>2.6</v>
       </c>
       <c r="F63" s="27" t="n">
         <v>-2715.19369056</v>
@@ -3539,14 +3545,14 @@
     <row r="64">
       <c r="B64" s="91">
         <f>B63+1</f>
-        <v/>
+        <v>87</v>
       </c>
       <c r="C64" s="92" t="n">
         <v>14233.47</v>
       </c>
       <c r="E64" s="26">
         <f>E63+0.1</f>
-        <v/>
+        <v>2.7</v>
       </c>
       <c r="F64" s="27" t="n">
         <v>3084.80630944</v>
@@ -3579,14 +3585,14 @@
     <row r="65">
       <c r="B65" s="91">
         <f>B64+1</f>
-        <v/>
+        <v>88</v>
       </c>
       <c r="C65" s="92" t="n">
         <v>12983.28</v>
       </c>
       <c r="E65" s="26">
         <f>E64+0.1</f>
-        <v/>
+        <v>2.8</v>
       </c>
       <c r="F65" s="27" t="n">
         <v>8884.80630944</v>
@@ -3619,14 +3625,14 @@
     <row r="66">
       <c r="B66" s="91">
         <f>B65+1</f>
-        <v/>
+        <v>89</v>
       </c>
       <c r="C66" s="92" t="n">
         <v>11733.09</v>
       </c>
       <c r="E66" s="26">
         <f>E65+0.1</f>
-        <v/>
+        <v>2.9</v>
       </c>
       <c r="F66" s="27" t="n">
         <v>14684.80630944</v>
@@ -3659,14 +3665,14 @@
     <row r="67">
       <c r="B67" s="93">
         <f>B66+1</f>
-        <v/>
+        <v>90</v>
       </c>
       <c r="C67" s="92" t="n">
         <v>10482.9</v>
       </c>
       <c r="E67" s="29">
         <f>E66+0.1</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="F67" s="27" t="n">
         <v>20484.80630944</v>
@@ -3699,14 +3705,14 @@
     <row r="68">
       <c r="B68" s="91">
         <f>B67+1</f>
-        <v/>
+        <v>91</v>
       </c>
       <c r="C68" s="92" t="n">
         <v>9232.709999999999</v>
       </c>
       <c r="E68" s="26">
         <f>E67+0.1</f>
-        <v/>
+        <v>3.1</v>
       </c>
       <c r="F68" s="27" t="n">
         <v>26284.80630944</v>
@@ -3739,14 +3745,14 @@
     <row r="69">
       <c r="B69" s="91">
         <f>B68+1</f>
-        <v/>
+        <v>92</v>
       </c>
       <c r="C69" s="92" t="n">
         <v>7982.52</v>
       </c>
       <c r="E69" s="26">
         <f>E68+0.1</f>
-        <v/>
+        <v>3.2</v>
       </c>
       <c r="F69" s="27" t="n">
         <v>32084.80630944</v>
@@ -3779,14 +3785,14 @@
     <row r="70">
       <c r="B70" s="91">
         <f>B69+1</f>
-        <v/>
+        <v>93</v>
       </c>
       <c r="C70" s="92" t="n">
         <v>6732.33</v>
       </c>
       <c r="E70" s="26">
         <f>E69+0.1</f>
-        <v/>
+        <v>3.3</v>
       </c>
       <c r="F70" s="27" t="n">
         <v>37884.80630944</v>
@@ -3819,14 +3825,14 @@
     <row r="71">
       <c r="B71" s="91">
         <f>B70+1</f>
-        <v/>
+        <v>94</v>
       </c>
       <c r="C71" s="92" t="n">
         <v>5482.14</v>
       </c>
       <c r="E71" s="26">
         <f>E70+0.1</f>
-        <v/>
+        <v>3.4</v>
       </c>
       <c r="F71" s="27" t="n">
         <v>43684.80630944</v>
@@ -3859,14 +3865,14 @@
     <row r="72">
       <c r="B72" s="91">
         <f>B71+1</f>
-        <v/>
+        <v>95</v>
       </c>
       <c r="C72" s="92" t="n">
         <v>4231.95</v>
       </c>
       <c r="E72" s="30">
         <f>E71+0.1</f>
-        <v/>
+        <v>3.5</v>
       </c>
       <c r="F72" s="31" t="n">
         <v>49484.80630944</v>
@@ -3899,7 +3905,7 @@
     <row r="73">
       <c r="B73" s="91">
         <f>B72+1</f>
-        <v/>
+        <v>96</v>
       </c>
       <c r="C73" s="92" t="n">
         <v>2981.76</v>
@@ -3908,7 +3914,7 @@
     <row r="74">
       <c r="B74" s="91">
         <f>B73+1</f>
-        <v/>
+        <v>97</v>
       </c>
       <c r="C74" s="92" t="n">
         <v>1731.57</v>
@@ -3917,7 +3923,7 @@
     <row r="75">
       <c r="B75" s="91">
         <f>B74+1</f>
-        <v/>
+        <v>98</v>
       </c>
       <c r="C75" s="92" t="n">
         <v>481.38</v>
@@ -3926,7 +3932,7 @@
     <row r="76">
       <c r="B76" s="91">
         <f>B75+1</f>
-        <v/>
+        <v>99</v>
       </c>
       <c r="C76" s="92" t="n">
         <v>-768.8099999999999</v>
@@ -3935,7 +3941,7 @@
     <row r="77">
       <c r="B77" s="91">
         <f>B76+1</f>
-        <v/>
+        <v>100</v>
       </c>
       <c r="C77" s="92" t="n">
         <v>-2019</v>
@@ -3944,7 +3950,7 @@
     <row r="78">
       <c r="B78" s="91">
         <f>B77+1</f>
-        <v/>
+        <v>101</v>
       </c>
       <c r="C78" s="92" t="n">
         <v>-3269.19</v>
@@ -3953,7 +3959,7 @@
     <row r="79">
       <c r="B79" s="91">
         <f>B78+1</f>
-        <v/>
+        <v>102</v>
       </c>
       <c r="C79" s="92" t="n">
         <v>-4519.38</v>
@@ -3962,7 +3968,7 @@
     <row r="80">
       <c r="B80" s="91">
         <f>B79+1</f>
-        <v/>
+        <v>103</v>
       </c>
       <c r="C80" s="92" t="n">
         <v>-5769.57</v>
@@ -3971,7 +3977,7 @@
     <row r="81">
       <c r="B81" s="91">
         <f>B80+1</f>
-        <v/>
+        <v>104</v>
       </c>
       <c r="C81" s="92" t="n">
         <v>-7019.76</v>
@@ -3980,25 +3986,25 @@
     <row r="82">
       <c r="B82" s="94">
         <f>B81+1</f>
-        <v/>
+        <v>105</v>
       </c>
       <c r="C82" s="95" t="n">
         <v>-8269.950000000001</v>
       </c>
     </row>
   </sheetData>
-  <scenarios>
-    <scenario name="Bieżący" locked="1" count="1">
+  <scenarios current="0" show="0" sqref="C6 D14 E14">
+    <scenario name="Bieżący" locked="1" count="3">
       <inputCells r="C6" val="3"/>
       <inputCells r="D14" val="15"/>
       <inputCells r="E14" val="80"/>
     </scenario>
-    <scenario name="Optymistyczny" locked="1" count="1">
+    <scenario name="Optymistyczny" locked="1" count="3">
       <inputCells r="C6" val="3.5"/>
       <inputCells r="D14" val="10"/>
       <inputCells r="E14" val="70"/>
     </scenario>
-    <scenario name="Pesymistyczny" locked="1" count="1">
+    <scenario name="Pesymistyczny" locked="1" count="3">
       <inputCells r="C6" val="2.5"/>
       <inputCells r="D14" val="20"/>
       <inputCells r="E14" val="90"/>

</xml_diff>

<commit_message>
E4-E6: zgodność ze schematem OOXML, poprawne style i komentarz LOOKUP
</commit_message>
<xml_diff>
--- a/E4-E6/TI.1_Excel.E4+E5+E6_PlikRoboczy.xlsx
+++ b/E4-E6/TI.1_Excel.E4+E5+E6_PlikRoboczy.xlsx
@@ -64,143 +64,143 @@
   </numFmts>
   <fonts count="20">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <charset val="238"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <charset val="238"/>
-      <family val="2"/>
-      <color rgb="FF9C0006"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b val="1"/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <charset val="238"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b val="1"/>
+      <u val="single"/>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <charset val="238"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color theme="1"/>
-      <sz val="12"/>
-      <u val="single"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b val="1"/>
+      <sz val="14"/>
+      <color theme="1"/>
       <name val="Times New Roman"/>
+      <family val="1"/>
       <charset val="238"/>
-      <family val="1"/>
-      <b val="1"/>
-      <color theme="1"/>
-      <sz val="14"/>
     </font>
     <font>
+      <b val="1"/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <charset val="238"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color rgb="FFFF0000"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b val="1"/>
+      <sz val="14"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <charset val="238"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color rgb="FFFF0000"/>
-      <sz val="14"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b val="1"/>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <charset val="238"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color rgb="FFFF0000"/>
-      <sz val="12"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b val="1"/>
+      <sz val="11"/>
+      <color rgb="FF00B0F0"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <charset val="238"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color rgb="FF00B0F0"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF00B0F0"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <charset val="238"/>
-      <family val="2"/>
-      <color rgb="FF00B0F0"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b val="1"/>
+      <sz val="12"/>
+      <color theme="5"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <charset val="238"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color theme="5"/>
-      <sz val="12"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <charset val="238"/>
-      <family val="2"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="9"/>
+      <color indexed="81"/>
       <name val="Tahoma"/>
+      <family val="2"/>
       <charset val="238"/>
-      <family val="2"/>
-      <color indexed="81"/>
-      <sz val="9"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
       <sz val="14"/>
+      <color rgb="FFFFFFFF"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="001F4E79"/>
+      <color rgb="FF1F4E79"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00006100"/>
+      <color rgb="FF006100"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00C00000"/>
+      <color rgb="FFC00000"/>
     </font>
     <font>
       <b val="1"/>
     </font>
     <font>
       <i val="1"/>
-      <color rgb="00595959"/>
       <sz val="9"/>
+      <color rgb="FF595959"/>
     </font>
   </fonts>
   <fills count="16">
@@ -280,12 +280,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
+        <fgColor rgb="FF1F4E79"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9D9D9"/>
+        <fgColor rgb="FFD9D9D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -912,16 +912,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </left>
       <right style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </right>
       <top style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </top>
       <bottom style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </bottom>
     </border>
   </borders>
@@ -1464,6 +1464,7 @@
       <text>
         <t>WYSZUKAJ (LOOKUP) zakłada dane posortowane rosnąco.
 Kolumna I36:I47 nie jest posortowana, więc wynik jest niewiarygodny.
+Próba: =LOOKUP(D51,I36:I47,B36:B47).
 Dlatego użyto INDEKS + PODAJ.POZYCJĘ.</t>
       </text>
     </comment>

</xml_diff>

<commit_message>
E6: wykres przebiegu w czasie, poprawki osi i etykiet wykresów
- dodany trzeci wykres (E6.2): liniowy przebieg kosztów całkowitych z kolumny Razem
- wykres kolumnowy: oś kategorii na dole, bezwzględne odwołania i cache serii
- wykres kołowy: etykiety procentowe z jednym miejscem po przecinku, linie odniesienia
- usunięta błędna walidacja danych w C7 (brak typu i formuły)
- wydruk: stałe skalowanie 90% i podziały stron, każdy wykres na osobnej stronie
</commit_message>
<xml_diff>
--- a/E4-E6/TI.1_Excel.E4+E5+E6_PlikRoboczy.xlsx
+++ b/E4-E6/TI.1_Excel.E4+E5+E6_PlikRoboczy.xlsx
@@ -47,7 +47,7 @@
     <definedName name="solver_typ" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_val" localSheetId="0" hidden="1">0</definedName>
     <definedName name="solver_ver" localSheetId="0" hidden="1">3</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Wykonalność'!$A$1:$N$135</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Wykonalność'!$A$1:$N$152</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Podsumowanie scenariuszy'!$A$1:$F$22</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -1156,84 +1156,268 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="pl-PL"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
           <a:bodyPr/>
+          <a:lstStyle/>
           <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
             <a:r>
+              <a:rPr lang="pl-PL"/>
               <a:t>Koszty składników w czasie (styczeń–grudzień)</a:t>
             </a:r>
           </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Wykonalność'!D35</f>
-            </strRef>
-          </tx>
-          <spPr>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Wykonalność'!$D$35</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Smocze sadło</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
             <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
-          </spPr>
-          <cat>
-            <strRef>
-              <f>'Wykonalność'!$B$36:$B$47</f>
-            </strRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Wykonalność'!$D$36:$D$47</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
-              <f>'Wykonalność'!E35</f>
-            </strRef>
-          </tx>
-          <spPr>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Wykonalność'!$B$36:$B$47</c:f>
+              <c:strCache>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>Sty</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Lut</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Kwi</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Maj</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Cze</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Lip</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Sie</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Wrz</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Paź</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Lis</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Gru</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Wykonalność'!$D$36:$D$47</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0</c:formatCode>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>1626.952703</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1952.343244</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2277.733784</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2603.124325</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2928.514866</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>3253.905406</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>650.7810813</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>325.3905406</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1626.952703</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1952.343244</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2277.733784</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2115.038514</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Wykonalność'!$E$35</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Mrówcze mięso</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
             <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
-          </spPr>
-          <cat>
-            <strRef>
-              <f>'Wykonalność'!$B$36:$B$47</f>
-            </strRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Wykonalność'!$E$36:$E$47</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="2"/>
-          <order val="2"/>
-          <tx>
-            <strRef>
-              <f>'Wykonalność'!F35</f>
-            </strRef>
-          </tx>
-          <spPr>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Wykonalność'!$B$36:$B$47</c:f>
+              <c:strCache>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>Sty</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Lut</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Kwi</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Maj</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Cze</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Lip</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Sie</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Wrz</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Paź</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Lis</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Gru</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Wykonalność'!$E$36:$E$47</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0</c:formatCode>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>5784.720722</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>6941.664867</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>8098.609011</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>9255.553156</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>10412.4973</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>11569.44144</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2313.888289</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1156.944144</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>5784.720722</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>6941.664867</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>8098.609011</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>7520.136939</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Wykonalność'!$F$35</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Makula-tura</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
             <a:solidFill>
               <a:srgbClr val="FFFF00"/>
             </a:solidFill>
@@ -1243,193 +1427,739 @@
               </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
-          </spPr>
-          <cat>
-            <strRef>
-              <f>'Wykonalność'!$B$36:$B$47</f>
-            </strRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Wykonalność'!$F$36:$F$47</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="3"/>
-          <order val="3"/>
-          <tx>
-            <strRef>
-              <f>'Wykonalność'!G35</f>
-            </strRef>
-          </tx>
-          <spPr>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Wykonalność'!$B$36:$B$47</c:f>
+              <c:strCache>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>Sty</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Lut</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Kwi</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Maj</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Cze</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Lip</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Sie</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Wrz</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Paź</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Lis</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Gru</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Wykonalność'!$F$36:$F$47</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0</c:formatCode>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>325.3905406</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>390.4686488</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>455.5467569</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>520.624865</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>585.7029731</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>650.7810813</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>130.1562163</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>65.07810813</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>325.3905406</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>390.4686488</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>455.5467569</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>423.0077028</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Wykonalność'!$G$35</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Magic Stufff</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
             <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
-          </spPr>
-          <cat>
-            <strRef>
-              <f>'Wykonalność'!$B$36:$B$47</f>
-            </strRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Wykonalność'!$G$36:$G$47</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="4"/>
-          <order val="4"/>
-          <tx>
-            <strRef>
-              <f>'Wykonalność'!H35</f>
-            </strRef>
-          </tx>
-          <spPr>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Wykonalność'!$B$36:$B$47</c:f>
+              <c:strCache>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>Sty</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Lut</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Kwi</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Maj</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Cze</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Lip</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Sie</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Wrz</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Paź</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Lis</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Gru</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Wykonalność'!$G$36:$G$47</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0</c:formatCode>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>45.19313064</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>54.23175677</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>63.2703829</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>72.30900903</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>81.34763516</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>90.38626129</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>18.07725226</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>9.038626129</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>45.19313064</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>54.23175677</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>63.2703829</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>58.75106984</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Wykonalność'!$H$35</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Woda</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
             <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
-          </spPr>
-          <cat>
-            <strRef>
-              <f>'Wykonalność'!$B$36:$B$47</f>
-            </strRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Wykonalność'!$H$36:$H$47</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="60"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Wykonalność'!$B$36:$B$47</c:f>
+              <c:strCache>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>Sty</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Lut</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Kwi</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Maj</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Cze</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Lip</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Sie</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Wrz</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Paź</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Lis</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Gru</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Wykonalność'!$H$36:$H$47</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0</c:formatCode>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>10.84635135</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>13.01562163</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>15.1848919</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>17.35416217</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>19.52343244</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>21.69270271</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>4.338540542</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2.169270271</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>10.84635135</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>13.01562163</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>15.1848919</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>14.10025676</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="60"/>
+        <c:overlap val="-10"/>
+        <c:axId val="10"/>
+        <c:axId val="100"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="10"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
               <a:bodyPr/>
+              <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
+                  <a:rPr lang="pl-PL"/>
                   <a:t>Miesiąc</a:t>
                 </a:r>
               </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="100"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="100"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:title>
+          <c:tx>
+            <c:rich>
               <a:bodyPr/>
+              <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
+                  <a:rPr lang="pl-PL"/>
                   <a:t>Koszt [€]</a:t>
                 </a:r>
               </a:p>
-            </rich>
-          </tx>
-        </title>
-        <numFmt formatCode="#,##0 &quot;€&quot;" sourceLinked="0"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="b"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="#,##0 &quot;€&quot;" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="10"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+</c:chartSpace>
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="pl-PL"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
           <a:bodyPr/>
+          <a:lstStyle/>
           <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
             <a:r>
+              <a:rPr lang="pl-PL"/>
               <a:t>Struktura rocznych kosztów składników</a:t>
             </a:r>
           </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <pieChart>
-        <varyColors val="1"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <spPr>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:pieChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Koszty roczne</c:v>
+          </c:tx>
+          <c:spPr>
             <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
-          </spPr>
-          <cat>
-            <strRef>
-              <f>'Wykonalność'!$D$35:$H$35</f>
-            </strRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Wykonalność'!$D$48:$H$48</f>
-            </numRef>
-          </val>
-        </ser>
-        <dLbls>
-          <dLblPos val="bestFit"/>
-          <showLegendKey val="0"/>
-          <showVal val="0"/>
-          <showCatName val="1"/>
-          <showSerName val="0"/>
-          <showPercent val="1"/>
-        </dLbls>
-        <firstSliceAng val="0"/>
-      </pieChart>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Wykonalność'!$D$35:$H$35</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>Smocze sadło</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Mrówcze mięso</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Makula-tura</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Magic Stufff</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Woda</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Wykonalność'!$D$48:$H$48</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>23590.8142</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>83878.45048</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4718.162839</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>655.3003943</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>157.2720946</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:dLbls>
+          <c:numFmt formatCode="0.0%" sourceLinked="0"/>
+          <c:dLblPos val="bestFit"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="1"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="1"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+        <c:firstSliceAng val="0"/>
+      </c:pieChart>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="pl-PL"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="pl-PL"/>
+              <a:t>Przebieg kosztów całkowitych w czasie (styczeń–grudzień)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Wykonalność'!$I$35</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Razem</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:srgbClr val="1F4E79"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="6"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="1F4E79"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Wykonalność'!$B$36:$B$47</c:f>
+              <c:strCache>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>Sty</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Lut</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Kwi</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Maj</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Cze</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Lip</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Sie</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Wrz</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Paź</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Lis</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Gru</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Wykonalność'!$I$36:$I$47</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0</c:formatCode>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>7793.103448</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>9351.724138</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>10910.34483</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>12468.96552</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>14027.58621</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>15586.2069</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>3117.241379</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1558.62069</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>7793.103448</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>9351.724138</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>10910.34483</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>10131.03448</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:marker val="1"/>
+        <c:axId val="10"/>
+        <c:axId val="100"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="10"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="pl-PL"/>
+                  <a:t>Miesiąc</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="100"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="100"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="pl-PL"/>
+                  <a:t>Koszt [€]</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="#,##0 &quot;€&quot;" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="10"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+</c:chartSpace>
 </file>
 
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1479,7 +2209,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -1519,6 +2249,28 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>131</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8640000" cy="3420000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1816,7 +2568,6 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A2:U82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -4026,18 +4777,19 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
-    <dataValidation sqref="C7" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" operator="lessThan"/>
+  <dataValidations count="1">
     <dataValidation sqref="C6" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="decimal" operator="greaterThan">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
-  <rowBreaks count="3" manualBreakCount="3">
+  <pageSetup orientation="landscape" paperSize="9" scale="90"/>
+  <rowBreaks count="5" manualBreakCount="5">
+    <brk id="32" min="0" max="16383" man="1"/>
     <brk id="58" min="0" max="16383" man="1"/>
     <brk id="83" min="0" max="16383" man="1"/>
     <brk id="104" min="0" max="16383" man="1"/>
+    <brk id="131" min="0" max="16383" man="1"/>
   </rowBreaks>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>